<commit_message>
adding experiment P data from Janice!
</commit_message>
<xml_diff>
--- a/data/constituents/raw_lab_data/phosphorus/Phosphorus_2023.xlsx
+++ b/data/constituents/raw_lab_data/phosphorus/Phosphorus_2023.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\huck4481\Documents\GitHub\hysteresis\data\raw_data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nicol\Documents\hysteresis\data\constituents\raw_lab_data\phosphorus\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29E391FD-6569-4E61-9013-B8007B2E14F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-25320" yWindow="360" windowWidth="25440" windowHeight="15270" xr2:uid="{5A712775-9F6B-46BF-88A1-72E8A328D28E}"/>
+    <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{5A712775-9F6B-46BF-88A1-72E8A328D28E}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>